<commit_message>
Fixing notation in the www/Lab6_Template.xlsx, addressing Phoebe Jackson's points.
</commit_message>
<xml_diff>
--- a/www/Lab6_Template.xlsx
+++ b/www/Lab6_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/CaptProton/GitRepos/LabRegression/www/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/CaptProton/GitRepos/JAC_PHYS/LabRegression/www/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFFEB78A-3668-764D-9432-1B4ADF60BC5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C74FD785-987B-1943-8444-97E1D148DE91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3260" yWindow="2160" windowWidth="28040" windowHeight="17440" xr2:uid="{978E5421-FC80-6446-9C13-B3201A983AFD}"/>
   </bookViews>
@@ -193,56 +193,6 @@
         <i/>
         <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>a</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="subscript"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> (m/s</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color theme="1"/>
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
@@ -261,10 +211,6 @@
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Effective acceleration
-</t>
-    </r>
-    <r>
       <rPr>
         <i/>
         <sz val="12"/>
@@ -272,16 +218,17 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
+      <t>𝜎</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <vertAlign val="subscript"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow (Body)"/>
+      </rPr>
       <t>a</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="subscript"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow (Body)"/>
-      </rPr>
-      <t>eff</t>
     </r>
     <r>
       <rPr>
@@ -315,6 +262,22 @@
   </si>
   <si>
     <r>
+      <t xml:space="preserve">Fractional mass difference
+</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>µ</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <rPr>
         <i/>
         <sz val="12"/>
@@ -322,7 +285,7 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>a</t>
+      <t>|a</t>
     </r>
     <r>
       <rPr>
@@ -332,7 +295,7 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t>2</t>
+      <t>+</t>
     </r>
     <r>
       <rPr>
@@ -341,7 +304,7 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t xml:space="preserve"> (m/s</t>
+      <t xml:space="preserve"> |(m/s</t>
     </r>
     <r>
       <rPr>
@@ -365,6 +328,146 @@
   </si>
   <si>
     <r>
+      <t>σ</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>a+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(m/s</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>|a</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>–</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>|(m/s</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>σ</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="subscript"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>a– </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>(m/s</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Average acceleration
+</t>
+    </r>
+    <r>
       <rPr>
         <i/>
         <sz val="12"/>
@@ -372,17 +475,16 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t>𝜎</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
+      <t>a</t>
+    </r>
+    <r>
+      <rPr>
         <vertAlign val="subscript"/>
         <sz val="12"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow (Body)"/>
       </rPr>
-      <t>a</t>
+      <t>av</t>
     </r>
     <r>
       <rPr>
@@ -410,108 +512,6 @@
         <rFont val="Aptos Narrow"/>
         <family val="2"/>
         <scheme val="minor"/>
-      </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Fractional mass difference
-</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>µ</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>σ</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="subscript"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>a1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>(m/s</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>σ</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="subscript"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>a2 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>(m/s</t>
-    </r>
-    <r>
-      <rPr>
-        <vertAlign val="superscript"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t>2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
       </rPr>
       <t>)</t>
     </r>
@@ -591,13 +591,25 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="32">
     <border>
@@ -938,7 +950,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1011,9 +1023,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
@@ -1021,114 +1030,135 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="centerContinuous" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1530,41 +1560,41 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="36" t="s">
+      <c r="B1" s="46"/>
+      <c r="C1" s="47" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="33"/>
-      <c r="E1" s="28" t="s">
+      <c r="D1" s="48"/>
+      <c r="E1" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="F1" s="3"/>
+      <c r="F1" s="50"/>
       <c r="H1" s="5" t="s">
         <v>3</v>
       </c>
       <c r="I1" s="6"/>
     </row>
     <row r="2" spans="1:26" s="1" customFormat="1" ht="20" x14ac:dyDescent="0.2">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="24" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="41" t="s">
-        <v>22</v>
-      </c>
-      <c r="D2" s="40" t="s">
+      <c r="B2" s="52" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="53" t="s">
+        <v>25</v>
+      </c>
+      <c r="D2" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="E2" s="55" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" s="56" t="s">
         <v>28</v>
-      </c>
-      <c r="E2" s="42" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="43" t="s">
-        <v>29</v>
       </c>
       <c r="H2" s="19" t="s">
         <v>1</v>
@@ -1599,12 +1629,12 @@
       </c>
     </row>
     <row r="3" spans="1:26" ht="19" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="37"/>
-      <c r="B3" s="38"/>
-      <c r="C3" s="45"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="44"/>
+      <c r="A3" s="32"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="38"/>
+      <c r="E3" s="33"/>
+      <c r="F3" s="34"/>
       <c r="H3" s="20" t="s">
         <v>2</v>
       </c>
@@ -1615,7 +1645,7 @@
         <f t="shared" ref="K3:K11" si="0">IF(ISNUMBER(C3),ABS(C3),NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="L3" s="26" t="e">
+      <c r="L3" s="25" t="e">
         <f t="shared" ref="L3:L11" si="1">IF(ISNUMBER(E3),ABS(E3),NA())</f>
         <v>#N/A</v>
       </c>
@@ -1623,11 +1653,11 @@
         <f t="shared" ref="M3:M11" si="2">IF(AND(ISNUMBER(A3), ISNUMBER($I$2)),ABS(A3/$I$2),NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="N3" s="26" t="e">
+      <c r="N3" s="25" t="e">
         <f>IF(ISNUMBER(AVERAGE(K3:L3)),AVERAGE(K3:L3),NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="O3" s="26" t="e">
+      <c r="O3" s="25" t="e">
         <f>IF(AND(ISNUMBER($A3),ISNUMBER($B3),ISNUMBER(I$3),ISNUMBER(I$2)),SQRT((B3/A3)^2 + ($I$3/$I$2)^2)*M3,NA())</f>
         <v>#N/A</v>
       </c>
@@ -1673,17 +1703,17 @@
       </c>
     </row>
     <row r="4" spans="1:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="29"/>
-      <c r="B4" s="25"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="34"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="30"/>
+      <c r="A4" s="26"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="36"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="27"/>
       <c r="K4" s="14" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
-      <c r="L4" s="26" t="e">
+      <c r="L4" s="25" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
@@ -1691,11 +1721,11 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="N4" s="26" t="e">
+      <c r="N4" s="25" t="e">
         <f t="shared" ref="N4:N11" si="7">IF(ISNUMBER(AVERAGE(K4:L4)),AVERAGE(K4:L4),NA())</f>
         <v>#N/A</v>
       </c>
-      <c r="O4" s="26" t="e">
+      <c r="O4" s="25" t="e">
         <f t="shared" ref="O4:O11" si="8">IF(AND(ISNUMBER($A4),ISNUMBER($B4),ISNUMBER(I$3),ISNUMBER(I$2)),SQRT((B4/A4)^2 + ($I$3/$I$2)^2)*M4,NA())</f>
         <v>#N/A</v>
       </c>
@@ -1741,12 +1771,12 @@
       </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A5" s="29"/>
-      <c r="B5" s="25"/>
-      <c r="C5" s="46"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="30"/>
+      <c r="A5" s="26"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="36"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="27"/>
       <c r="H5" s="5" t="s">
         <v>4</v>
       </c>
@@ -1755,7 +1785,7 @@
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
-      <c r="L5" s="26" t="e">
+      <c r="L5" s="25" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
@@ -1763,11 +1793,11 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="N5" s="26" t="e">
+      <c r="N5" s="25" t="e">
         <f t="shared" si="7"/>
         <v>#N/A</v>
       </c>
-      <c r="O5" s="26" t="e">
+      <c r="O5" s="25" t="e">
         <f t="shared" si="8"/>
         <v>#N/A</v>
       </c>
@@ -1813,12 +1843,12 @@
       </c>
     </row>
     <row r="6" spans="1:26" ht="20" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="29"/>
-      <c r="B6" s="25"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="34"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="30"/>
+      <c r="A6" s="26"/>
+      <c r="B6" s="24"/>
+      <c r="C6" s="36"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="27"/>
       <c r="H6" s="21" t="s">
         <v>5</v>
       </c>
@@ -1829,7 +1859,7 @@
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
-      <c r="L6" s="26" t="e">
+      <c r="L6" s="25" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
@@ -1837,11 +1867,11 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="N6" s="26" t="e">
+      <c r="N6" s="25" t="e">
         <f t="shared" si="7"/>
         <v>#N/A</v>
       </c>
-      <c r="O6" s="26" t="e">
+      <c r="O6" s="25" t="e">
         <f t="shared" si="8"/>
         <v>#N/A</v>
       </c>
@@ -1887,17 +1917,17 @@
       </c>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A7" s="29"/>
-      <c r="B7" s="25"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="25"/>
-      <c r="F7" s="30"/>
+      <c r="A7" s="26"/>
+      <c r="B7" s="24"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="27"/>
       <c r="K7" s="14" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
-      <c r="L7" s="26" t="e">
+      <c r="L7" s="25" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
@@ -1905,11 +1935,11 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="N7" s="26" t="e">
+      <c r="N7" s="25" t="e">
         <f t="shared" si="7"/>
         <v>#N/A</v>
       </c>
-      <c r="O7" s="26" t="e">
+      <c r="O7" s="25" t="e">
         <f t="shared" si="8"/>
         <v>#N/A</v>
       </c>
@@ -1955,17 +1985,17 @@
       </c>
     </row>
     <row r="8" spans="1:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="29"/>
-      <c r="B8" s="25"/>
-      <c r="C8" s="46"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="25"/>
-      <c r="F8" s="30"/>
+      <c r="A8" s="26"/>
+      <c r="B8" s="24"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="27"/>
       <c r="K8" s="14" t="e">
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
-      <c r="L8" s="26" t="e">
+      <c r="L8" s="25" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
@@ -1973,11 +2003,11 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="N8" s="26" t="e">
+      <c r="N8" s="25" t="e">
         <f t="shared" si="7"/>
         <v>#N/A</v>
       </c>
-      <c r="O8" s="26" t="e">
+      <c r="O8" s="25" t="e">
         <f t="shared" si="8"/>
         <v>#N/A</v>
       </c>
@@ -2023,12 +2053,12 @@
       </c>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A9" s="29"/>
-      <c r="B9" s="25"/>
-      <c r="C9" s="46"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="25"/>
-      <c r="F9" s="30"/>
+      <c r="A9" s="26"/>
+      <c r="B9" s="24"/>
+      <c r="C9" s="36"/>
+      <c r="D9" s="30"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="27"/>
       <c r="H9" s="2" t="s">
         <v>6</v>
       </c>
@@ -2037,7 +2067,7 @@
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
-      <c r="L9" s="26" t="e">
+      <c r="L9" s="25" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
@@ -2045,11 +2075,11 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="N9" s="26" t="e">
+      <c r="N9" s="25" t="e">
         <f t="shared" si="7"/>
         <v>#N/A</v>
       </c>
-      <c r="O9" s="26" t="e">
+      <c r="O9" s="25" t="e">
         <f t="shared" si="8"/>
         <v>#N/A</v>
       </c>
@@ -2095,12 +2125,12 @@
       </c>
     </row>
     <row r="10" spans="1:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="29"/>
-      <c r="B10" s="25"/>
-      <c r="C10" s="46"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="25"/>
-      <c r="F10" s="30"/>
+      <c r="A10" s="26"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="36"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="27"/>
       <c r="H10" s="22" t="str">
         <f>IF(NOT(ISNUMBER(I2)), "No Mtot", IF(SUM(R:R)&gt;=5, "Okay", "Too few data points"))</f>
         <v>No Mtot</v>
@@ -2110,7 +2140,7 @@
         <f t="shared" si="0"/>
         <v>#N/A</v>
       </c>
-      <c r="L10" s="26" t="e">
+      <c r="L10" s="25" t="e">
         <f t="shared" si="1"/>
         <v>#N/A</v>
       </c>
@@ -2118,11 +2148,11 @@
         <f t="shared" si="2"/>
         <v>#N/A</v>
       </c>
-      <c r="N10" s="26" t="e">
+      <c r="N10" s="25" t="e">
         <f t="shared" si="7"/>
         <v>#N/A</v>
       </c>
-      <c r="O10" s="26" t="e">
+      <c r="O10" s="25" t="e">
         <f t="shared" si="8"/>
         <v>#N/A</v>
       </c>
@@ -2168,11 +2198,11 @@
       </c>
     </row>
     <row r="11" spans="1:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="31"/>
-      <c r="B11" s="32"/>
-      <c r="C11" s="47"/>
-      <c r="D11" s="35"/>
-      <c r="E11" s="32"/>
+      <c r="A11" s="28"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="37"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="29"/>
       <c r="F11" s="12"/>
       <c r="K11" s="16" t="e">
         <f t="shared" si="0"/>
@@ -2248,193 +2278,193 @@
     </row>
     <row r="15" spans="1:26" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="16" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="B16" s="28"/>
-      <c r="C16" s="27" t="s">
+      <c r="B16" s="58"/>
+      <c r="C16" s="59" t="s">
         <v>19</v>
       </c>
-      <c r="D16" s="3"/>
+      <c r="D16" s="60"/>
     </row>
     <row r="17" spans="1:4" ht="55" x14ac:dyDescent="0.2">
-      <c r="A17" s="51" t="s">
-        <v>27</v>
-      </c>
-      <c r="B17" s="54" t="s">
+      <c r="A17" s="61" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="52" t="s">
+      <c r="B17" s="62" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="63" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17" s="64" t="s">
         <v>23</v>
-      </c>
-      <c r="D17" s="53" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="7" t="str">
-        <f>IF(ISNUMBER(M3),M3,"")</f>
-        <v/>
-      </c>
-      <c r="B18" s="55" t="str">
-        <f>IF(ISNUMBER(N3),N3,"")</f>
+        <f t="shared" ref="A18:A26" si="11">IF(ISNUMBER(M3),M3,"")</f>
+        <v/>
+      </c>
+      <c r="B18" s="41" t="str">
+        <f t="shared" ref="B18:B26" si="12">IF(ISNUMBER(N3),N3,"")</f>
         <v/>
       </c>
       <c r="C18" s="4" t="str">
-        <f>IF(ISNUMBER(O3),O3,"")</f>
-        <v/>
-      </c>
-      <c r="D18" s="57" t="str">
-        <f>IF(ISNUMBER(P3),P3,"")</f>
+        <f t="shared" ref="C18:C26" si="13">IF(ISNUMBER(O3),O3,"")</f>
+        <v/>
+      </c>
+      <c r="D18" s="43" t="str">
+        <f t="shared" ref="D18:D26" si="14">IF(ISNUMBER(P3),P3,"")</f>
         <v/>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="7" t="str">
-        <f>IF(ISNUMBER(M4),M4,"")</f>
-        <v/>
-      </c>
-      <c r="B19" s="55" t="str">
-        <f>IF(ISNUMBER(N4),N4,"")</f>
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="B19" s="41" t="str">
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="C19" s="4" t="str">
-        <f>IF(ISNUMBER(O4),O4,"")</f>
-        <v/>
-      </c>
-      <c r="D19" s="57" t="str">
-        <f>IF(ISNUMBER(P4),P4,"")</f>
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="D19" s="43" t="str">
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="7" t="str">
-        <f>IF(ISNUMBER(M5),M5,"")</f>
-        <v/>
-      </c>
-      <c r="B20" s="55" t="str">
-        <f>IF(ISNUMBER(N5),N5,"")</f>
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="B20" s="41" t="str">
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="C20" s="4" t="str">
-        <f>IF(ISNUMBER(O5),O5,"")</f>
-        <v/>
-      </c>
-      <c r="D20" s="57" t="str">
-        <f>IF(ISNUMBER(P5),P5,"")</f>
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="D20" s="43" t="str">
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="7" t="str">
-        <f>IF(ISNUMBER(M6),M6,"")</f>
-        <v/>
-      </c>
-      <c r="B21" s="55" t="str">
-        <f>IF(ISNUMBER(N6),N6,"")</f>
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="B21" s="41" t="str">
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="C21" s="4" t="str">
-        <f>IF(ISNUMBER(O6),O6,"")</f>
-        <v/>
-      </c>
-      <c r="D21" s="57" t="str">
-        <f>IF(ISNUMBER(P6),P6,"")</f>
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="D21" s="43" t="str">
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" s="7" t="str">
-        <f>IF(ISNUMBER(M7),M7,"")</f>
-        <v/>
-      </c>
-      <c r="B22" s="55" t="str">
-        <f>IF(ISNUMBER(N7),N7,"")</f>
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="B22" s="41" t="str">
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="C22" s="4" t="str">
-        <f>IF(ISNUMBER(O7),O7,"")</f>
-        <v/>
-      </c>
-      <c r="D22" s="57" t="str">
-        <f>IF(ISNUMBER(P7),P7,"")</f>
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="D22" s="43" t="str">
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" s="7" t="str">
-        <f>IF(ISNUMBER(M8),M8,"")</f>
-        <v/>
-      </c>
-      <c r="B23" s="55" t="str">
-        <f>IF(ISNUMBER(N8),N8,"")</f>
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="B23" s="41" t="str">
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="C23" s="4" t="str">
-        <f>IF(ISNUMBER(O8),O8,"")</f>
-        <v/>
-      </c>
-      <c r="D23" s="57" t="str">
-        <f>IF(ISNUMBER(P8),P8,"")</f>
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="D23" s="43" t="str">
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" s="7" t="str">
-        <f>IF(ISNUMBER(M9),M9,"")</f>
-        <v/>
-      </c>
-      <c r="B24" s="55" t="str">
-        <f>IF(ISNUMBER(N9),N9,"")</f>
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="B24" s="41" t="str">
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="C24" s="4" t="str">
-        <f>IF(ISNUMBER(O9),O9,"")</f>
-        <v/>
-      </c>
-      <c r="D24" s="57" t="str">
-        <f>IF(ISNUMBER(P9),P9,"")</f>
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="D24" s="43" t="str">
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="7" t="str">
-        <f>IF(ISNUMBER(M10),M10,"")</f>
-        <v/>
-      </c>
-      <c r="B25" s="55" t="str">
-        <f>IF(ISNUMBER(N10),N10,"")</f>
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="B25" s="41" t="str">
+        <f t="shared" si="12"/>
         <v/>
       </c>
       <c r="C25" s="4" t="str">
-        <f>IF(ISNUMBER(O10),O10,"")</f>
-        <v/>
-      </c>
-      <c r="D25" s="57" t="str">
-        <f>IF(ISNUMBER(P10),P10,"")</f>
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="D25" s="43" t="str">
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
     <row r="26" spans="1:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="49" t="str">
-        <f>IF(ISNUMBER(M11),M11,"")</f>
-        <v/>
-      </c>
-      <c r="B26" s="56" t="str">
-        <f>IF(ISNUMBER(N11),N11,"")</f>
-        <v/>
-      </c>
-      <c r="C26" s="50" t="str">
-        <f>IF(ISNUMBER(O11),O11,"")</f>
-        <v/>
-      </c>
-      <c r="D26" s="58" t="str">
-        <f>IF(ISNUMBER(P11),P11,"")</f>
+      <c r="A26" s="39" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="B26" s="42" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="C26" s="40" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="D26" s="44" t="str">
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="DMbPQZ6B0AhfTbJStIT+cVwPogB68LJC+EOZ8jkthmC+mgrCQGf8Jtj0Wf5L4idNEUcGRckbii72Wk6aHmF1YQ==" saltValue="uQQcjjdv2buAsIQqBvhixA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="BCQ128nO+7nAunQWTZuDQEJj3vL6Vxou4x7r/eTihG1eOHMprw/4ftZvho/Up76A2WiVGYMa6Qn3tYO/VqGAcQ==" saltValue="h0+dKS3+7Nxt/+NfbwE7eg==" spinCount="100000" sheet="1" objects="1" scenarios="1" formatCells="0"/>
   <conditionalFormatting sqref="A3:F11">
     <cfRule type="expression" dxfId="4" priority="9">
       <formula>U3&gt;0</formula>

</xml_diff>